<commit_message>
Add course plans and program details for various subjects at Dalarna University
- Created new course plans for unknown subjects (GV, M, V) under the IIT department.
- Added MOC page for "Okänt ämne" with links to the new courses.
- Introduced a stray MOC page for "Stray Okänt ämne" detailing stray courses in the IIT department.
- Added course plan for "Missbruk och beroende" (GSA2XN) under the IHV department.
- Created program details for the "Ämneslärarprogrammet årskurs 7-9" (L7I9A) under the IKS department.
- Added course plans for "Språk-, läs- och skrivdidaktisk fördjupning" for grades 1-3 (ASV2CP) and 4-6 (ASV2CQ) under the ISLL department.
- Created a placeholder for the VVA program.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Omfång på lärandemål.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Omfång på lärandemål.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Omfång på lärandemål" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Omfång på lärandemål'!$A$1:$E$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Omfång på lärandemål'!$A$1:$E$225</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E224"/>
+  <dimension ref="A1:E225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4495,7 +4495,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4510,19 +4510,19 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>18 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GSA352</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4537,19 +4537,19 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>18 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA352</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>GSA3DM</t>
+          <t>GSA352</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4564,12 +4564,12 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>23 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA352</t>
         </is>
       </c>
     </row>
@@ -4586,12 +4586,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>28 ord: - visa förmåga att på grundläggande nivå tillämpa metoder i socialt arbete inom …</t>
+          <t>23 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>27 ord: - kunna redogöra för grundläggande metoder och arbetssätt som tillämpas i social…</t>
+          <t>28 ord: - visa förmåga att på grundläggande nivå tillämpa metoder i socialt arbete inom …</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -4630,7 +4630,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GSA3DN</t>
+          <t>GSA3DM</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4640,17 +4640,17 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>27 ord: - kunna redogöra för grundläggande metoder och arbetssätt som tillämpas i social…</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DM</t>
         </is>
       </c>
     </row>
@@ -4667,12 +4667,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>29 ord: - visa förmåga att reflektera över hur de egna personliga värderingarna avseende…</t>
+          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
@@ -4684,7 +4684,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>GSA3DP</t>
+          <t>GSA3DN</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4694,24 +4694,24 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>29 ord: - visa förmåga att reflektera över hur de egna personliga värderingarna avseende…</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>GSA3DQ</t>
+          <t>GSA3DP</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4726,12 +4726,12 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>14 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DP</t>
         </is>
       </c>
     </row>
@@ -4748,12 +4748,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>27 ord: - redogöra för perspektiv på och metoder för socialt arbete med barn, familjer, …</t>
+          <t>14 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
@@ -4780,7 +4780,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>27 ord: - visa förmåga att reflektera över hur de egna personliga värderingarna rörande …</t>
+          <t>27 ord: - redogöra för perspektiv på och metoder för socialt arbete med barn, familjer, …</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
@@ -4792,7 +4792,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GSA3DR</t>
+          <t>GSA3DQ</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4802,24 +4802,24 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>27 ord: - visa förmåga att reflektera över hur de egna personliga värderingarna rörande …</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DQ</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GSA3DS</t>
+          <t>GSA3DR</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4834,19 +4834,19 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>18 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DR</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GSA3FK</t>
+          <t>GSA3DS</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4861,12 +4861,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>18 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3FK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
         </is>
       </c>
     </row>
@@ -4883,12 +4883,12 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>34 ord: - utifrån ett brukarperspektiv genomföra olika typer av utredningar inom socialt…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
@@ -4900,7 +4900,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GSA3FL</t>
+          <t>GSA3FK</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4910,24 +4910,24 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>18 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>34 ord: - utifrån ett brukarperspektiv genomföra olika typer av utredningar inom socialt…</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3FL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3FK</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GSA3HA</t>
+          <t>GSA3FL</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4942,19 +4942,19 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>18 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3HA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3FL</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>SA1045</t>
+          <t>GSA3HA</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4969,19 +4969,19 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1045</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3HA</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>SA1048</t>
+          <t>SA1045</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4996,12 +4996,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>23 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1048</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1045</t>
         </is>
       </c>
     </row>
@@ -5018,12 +5018,12 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>28 ord: - visa förmåga att på grundläggande nivå tillämpa metoder i socialt arbete inom …</t>
+          <t>23 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>27 ord: - kunna redogöra för grundläggande metoder och arbetssätt som tillämpas i social…</t>
+          <t>28 ord: - visa förmåga att på grundläggande nivå tillämpa metoder i socialt arbete inom …</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
@@ -5062,7 +5062,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>SA2020</t>
+          <t>SA1048</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -5072,17 +5072,17 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>26 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
+          <t>27 ord: - kunna redogöra för grundläggande metoder och arbetssätt som tillämpas i social…</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA1048</t>
         </is>
       </c>
     </row>
@@ -5099,12 +5099,12 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>32 ord: - uppvisa kunskaper som utgör innehåll i en tolkningsram (till exempel teori, te…</t>
+          <t>26 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>32 ord: - analysera resultat från ett vetenskapligt arbete på sådant sätt att tolkningsr…</t>
+          <t>32 ord: - uppvisa kunskaper som utgör innehåll i en tolkningsram (till exempel teori, te…</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>32 ord: - komponera och integrera de olika delarna i ett vetenskapligt arbete på ett såd…</t>
+          <t>32 ord: - analysera resultat från ett vetenskapligt arbete på sådant sätt att tolkningsr…</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -5170,7 +5170,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>SA3008</t>
+          <t>SA2020</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -5180,17 +5180,17 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>13 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>32 ord: - komponera och integrera de olika delarna i ett vetenskapligt arbete på ett såd…</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA3008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA2020</t>
         </is>
       </c>
     </row>
@@ -5207,12 +5207,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>30 ord: - komponera och integrera de olika delarna i ett vetenskapligt arbete på ett såd…</t>
+          <t>13 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -5224,12 +5224,12 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>ASR24V</t>
+          <t>SA3008</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -5239,12 +5239,12 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>26 ord: - redogöra för centrala begrepp inom global sexuell och reproduktiv hälsa och rä…</t>
+          <t>30 ord: - komponera och integrera de olika delarna i ett vetenskapligt arbete på ett såd…</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR24V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SA3008</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>27 ord: - ur ett rättighetsperspektiv analysera och diskutera hur sociala, ekonomiska, m…</t>
+          <t>26 ord: - redogöra för centrala begrepp inom global sexuell och reproduktiv hälsa och rä…</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
@@ -5278,7 +5278,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>ASR25P</t>
+          <t>ASR24V</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -5293,19 +5293,19 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>28 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av o…</t>
+          <t>27 ord: - ur ett rättighetsperspektiv analysera och diskutera hur sociala, ekonomiska, m…</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR24V</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>ASR26N</t>
+          <t>ASR25P</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -5315,17 +5315,17 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>11 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>28 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av o…</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25P</t>
         </is>
       </c>
     </row>
@@ -5342,12 +5342,12 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>30 ord: - diskutera vikten av samarbete och lagarbete inom och mellan utbildningsinstitu…</t>
+          <t>11 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -5359,7 +5359,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>ASR26N</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -5374,19 +5374,19 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
+          <t>30 ord: - diskutera vikten av samarbete och lagarbete inom och mellan utbildningsinstitu…</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -5396,17 +5396,17 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
+          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
+          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
+          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
@@ -5467,7 +5467,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>ASR29S</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5482,19 +5482,19 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>27 ord: - analysera och värdera resultat i relation till tidigare forskning, värdera den…</t>
+          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>ASR29T</t>
+          <t>ASR29S</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5509,12 +5509,12 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>26 ord: - problematisera och reflektera över kvinnans, barnets och närståendes roller oc…</t>
+          <t>27 ord: - analysera och värdera resultat i relation till tidigare forskning, värdera den…</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29S</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>28 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av o…</t>
+          <t>26 ord: - problematisera och reflektera över kvinnans, barnets och närståendes roller oc…</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
@@ -5548,7 +5548,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>ASR29T</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5563,19 +5563,19 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>26 ord: - i simulerad miljö utföra undersökningar och behandlingar vid komplicerad gravi…</t>
+          <t>28 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av o…</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29T</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>ASR29V</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5585,17 +5585,17 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
+          <t>26 ord: - i simulerad miljö utföra undersökningar och behandlingar vid komplicerad gravi…</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
@@ -5612,12 +5612,12 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
+          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
@@ -5644,7 +5644,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
+          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
@@ -5656,7 +5656,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>ASR29W</t>
+          <t>ASR29V</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5671,19 +5671,19 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
+          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29V</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>ASR2AD</t>
+          <t>ASR29W</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5698,19 +5698,19 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>28 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av k…</t>
+          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2AD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29W</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>ASR2BM</t>
+          <t>ASR2AD</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5720,24 +5720,24 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>28 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av k…</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2BM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2AD</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>ASR2CE</t>
+          <t>ASR2BM</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5747,24 +5747,24 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>26 ord: - redogöra för centrala begrepp inom global sexuell och reproduktiv hälsa och rä…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2BM</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>GSR38B</t>
+          <t>ASR2CE</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5779,19 +5779,19 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>33 ord: - uppvisa kunskap, förståelse och reflekterande färdigheter om sexuell och repro…</t>
+          <t>26 ord: - redogöra för centrala begrepp inom global sexuell och reproduktiv hälsa och rä…</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CE</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>SR3001</t>
+          <t>GSR38B</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5806,19 +5806,19 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>30 ord: - värdera olika strategier för ledarskap och interventioner som har potential at…</t>
+          <t>33 ord: - uppvisa kunskap, förståelse och reflekterande färdigheter om sexuell och repro…</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>SR3002</t>
+          <t>SR3001</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5833,19 +5833,19 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>27 ord: - analysera och kritiskt värdera styrkor och svagheter i forskningsprocessens ol…</t>
+          <t>30 ord: - värdera olika strategier för ledarskap och interventioner som har potential at…</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>SR3007</t>
+          <t>SR3002</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5855,24 +5855,24 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>12 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>27 ord: - analysera och kritiskt värdera styrkor och svagheter i forskningsprocessens ol…</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3002</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>SR3008</t>
+          <t>SR3007</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5887,19 +5887,19 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>12 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3007</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>SR3009</t>
+          <t>SR3008</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5909,17 +5909,17 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>26 ord: - analysera betydelsen av hälsofrämjande arbete under den reproduktiva livscykel…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3008</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>29 ord: - identifiera problemområden och formulera relevanta frågeställningar som rör gr…</t>
+          <t>26 ord: - analysera betydelsen av hälsofrämjande arbete under den reproduktiva livscykel…</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>27 ord: - redogöra för benigna och maligna gynekologiska förändringar, värdera hälsotill…</t>
+          <t>29 ord: - identifiera problemområden och formulera relevanta frågeställningar som rör gr…</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
@@ -5980,7 +5980,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>SR3010</t>
+          <t>SR3009</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5995,19 +5995,19 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>27 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av g…</t>
+          <t>27 ord: - redogöra för benigna och maligna gynekologiska förändringar, värdera hälsotill…</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>SR3011</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -6022,19 +6022,19 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
+          <t>27 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av g…</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>SR3012</t>
+          <t>SR3011</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -6044,17 +6044,17 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
+          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3011</t>
         </is>
       </c>
     </row>
@@ -6071,12 +6071,12 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
+          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
+          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
@@ -6115,7 +6115,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>SR3014</t>
+          <t>SR3012</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -6125,17 +6125,17 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>11 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
+          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
         </is>
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3012</t>
         </is>
       </c>
     </row>
@@ -6152,12 +6152,12 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>30 ord: - med ett professionellt förhållningssätt informera, ge stöd och trygghet i dial…</t>
+          <t>11 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
@@ -6169,7 +6169,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>SR3015</t>
+          <t>SR3014</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -6179,17 +6179,17 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>14 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
+          <t>30 ord: - med ett professionellt förhållningssätt informera, ge stöd och trygghet i dial…</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3014</t>
         </is>
       </c>
     </row>
@@ -6206,12 +6206,12 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>35 ord: - självständigt handlägga preventivmedelsrådgivning och informera om lämpliga an…</t>
+          <t>14 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
@@ -6238,7 +6238,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>26 ord: - kritiskt analysera, värdera, föreslå och följa upp vårdnadsinsatser och behand…</t>
+          <t>35 ord: - självständigt handlägga preventivmedelsrådgivning och informera om lämpliga an…</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
@@ -6250,12 +6250,12 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>AVV2A6</t>
+          <t>SR3015</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>VÅE</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -6265,19 +6265,19 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>26 ord: - kritiskt reflektera över hur kvalitets- och säkerhetsledning organiseras och r…</t>
+          <t>26 ord: - kritiskt analysera, värdera, föreslå och följa upp vårdnadsinsatser och behand…</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV2A6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3015</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>VV2002</t>
+          <t>AVV2A6</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -6292,19 +6292,19 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>29 ord: - redogöra för gällande regelverk för olika professioner inom kommunal äldreomso…</t>
+          <t>26 ord: - kritiskt reflektera över hur kvalitets- och säkerhetsledning organiseras och r…</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV2002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV2A6</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>VV3006</t>
+          <t>VV2002</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -6314,24 +6314,24 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>29 ord: - redogöra för gällande regelverk för olika professioner inom kommunal äldreomso…</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV2002</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>VV3011</t>
+          <t>VV3006</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -6346,19 +6346,19 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>19 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3006</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>VV3012</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -6368,17 +6368,17 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa adekvat vetenskaplig design och metod i datainsamling och analys samt…</t>
+          <t>19 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
@@ -6400,7 +6400,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>29 ord: - analysera och värdera resultat i relation till tidigare forskning samt den kli…</t>
+          <t>29 ord: - tillämpa adekvat vetenskaplig design och metod i datainsamling och analys samt…</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
@@ -6412,7 +6412,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>VV3017</t>
+          <t>VV3012</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -6427,12 +6427,12 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa adekvat vetenskaplig design och metod i datainsamling och analys samt…</t>
+          <t>29 ord: - analysera och värdera resultat i relation till tidigare forskning samt den kli…</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3012</t>
         </is>
       </c>
     </row>
@@ -6454,7 +6454,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>29 ord: - analysera och värdera resultat i relation till tidigare forskning samt den kli…</t>
+          <t>29 ord: - tillämpa adekvat vetenskaplig design och metod i datainsamling och analys samt…</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -6481,17 +6481,44 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
+          <t>29 ord: - analysera och värdera resultat i relation till tidigare forskning samt den kli…</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>VV3017</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>VÅE</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
           <t>26 ord: - göra relevanta bedömningar på mikro-, meso- och makronivå med hänsyn till samh…</t>
         </is>
       </c>
-      <c r="E224" s="2" t="inlineStr">
+      <c r="E225" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E224"/>
+  <autoFilter ref="A1:E225"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -6939,6 +6966,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E223" r:id="rId444"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A224" r:id="rId445"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E224" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A225" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E225" r:id="rId448"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans and related documents for ISLL and IHV programs
- Modified course plan documents for Kinesiska, Svenska som andraspråk, and Omvårdnad, including updates to course names, tags, and learning outcomes.
- Added new course plans for "Handledning inom omvårdnad vid Verksamhetsförlagd utbildning (VFU)" and "Graviditet, förlossning och postpartumperiod I & II".
- Updated the number of courses and their descriptions in MOC documents to reflect current offerings.
- Adjusted download links and file references in markdown files to ensure accuracy.
- Revised binary files for various analyses and course plans to reflect recent changes.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Omfång på lärandemål.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Omfång på lärandemål.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Omfång på lärandemål" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Omfång på lärandemål'!$A$1:$E$207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Omfång på lärandemål'!$A$1:$E$209</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E207"/>
+  <dimension ref="A1:E209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5224,7 +5224,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>GSR38B</t>
+          <t>ASR2CS</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -5234,24 +5234,24 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>33 ord: - uppvisa kunskap, förståelse och reflekterande färdigheter om sexuell och repro…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CS</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>SR3001</t>
+          <t>ASR2CS</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -5266,19 +5266,19 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>30 ord: - värdera olika strategier för ledarskap och interventioner som har potential at…</t>
+          <t>26 ord: - redogöra för och motivera metoder för att främja, undersöka och övervaka kvinn…</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR2CS</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>SR3002</t>
+          <t>GSR38B</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -5293,19 +5293,19 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>27 ord: - analysera och kritiskt värdera styrkor och svagheter i forskningsprocessens ol…</t>
+          <t>33 ord: - uppvisa kunskap, förståelse och reflekterande färdigheter om sexuell och repro…</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>SR3007</t>
+          <t>SR3001</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -5315,24 +5315,24 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>12 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>30 ord: - värdera olika strategier för ledarskap och interventioner som har potential at…</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3001</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>SR3008</t>
+          <t>SR3002</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -5342,24 +5342,24 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>27 ord: - analysera och kritiskt värdera styrkor och svagheter i forskningsprocessens ol…</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3002</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>SR3009</t>
+          <t>SR3007</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -5369,24 +5369,24 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>26 ord: - analysera betydelsen av hälsofrämjande arbete under den reproduktiva livscykel…</t>
+          <t>12 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3007</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>SR3009</t>
+          <t>SR3008</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -5396,17 +5396,17 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>29 ord: - identifiera problemområden och formulera relevanta frågeställningar som rör gr…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3008</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>27 ord: - redogöra för benigna och maligna gynekologiska förändringar, värdera hälsotill…</t>
+          <t>26 ord: - analysera betydelsen av hälsofrämjande arbete under den reproduktiva livscykel…</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -5440,7 +5440,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>SR3010</t>
+          <t>SR3009</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -5455,19 +5455,19 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>27 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av g…</t>
+          <t>29 ord: - identifiera problemområden och formulera relevanta frågeställningar som rör gr…</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>SR3011</t>
+          <t>SR3009</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5482,19 +5482,19 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
+          <t>27 ord: - redogöra för benigna och maligna gynekologiska förändringar, värdera hälsotill…</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3009</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>SR3012</t>
+          <t>SR3010</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5504,24 +5504,24 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
+          <t>27 ord: - i simulerad miljö utföra undersökningar och behandlingar vid handläggning av g…</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3010</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>SR3012</t>
+          <t>SR3011</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5536,12 +5536,12 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
+          <t>26 ord: - aktivt delta i vård av kvinnor med normal graviditet inför, under och efter fö…</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3011</t>
         </is>
       </c>
     </row>
@@ -5558,12 +5558,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
+          <t>13 lärandemål (maximum rekommenderat: 10 för 9 hp)</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
@@ -5575,7 +5575,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>SR3014</t>
+          <t>SR3012</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5585,24 +5585,24 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>11 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
+          <t>26 ord: - aktivt delta i abortverksamhet och visa på självständighet i vården av kvinnor…</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3012</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>SR3014</t>
+          <t>SR3012</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5617,19 +5617,19 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>30 ord: - med ett professionellt förhållningssätt informera, ge stöd och trygghet i dial…</t>
+          <t>29 ord: - tillämpa ett professionellt förhållningssätt i kommunikation med vårdtagare oc…</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3012</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>SR3015</t>
+          <t>SR3014</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5644,19 +5644,19 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>14 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
+          <t>11 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3014</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>SR3015</t>
+          <t>SR3014</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>35 ord: - självständigt handlägga preventivmedelsrådgivning och informera om lämpliga an…</t>
+          <t>30 ord: - med ett professionellt förhållningssätt informera, ge stöd och trygghet i dial…</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3014</t>
         </is>
       </c>
     </row>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>26 ord: - kritiskt analysera, värdera, föreslå och följa upp vårdnadsinsatser och behand…</t>
+          <t>14 lärandemål (maximum rekommenderat: 10 för 13.5 hp)</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -5710,12 +5710,12 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>AVV2A6</t>
+          <t>SR3015</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>VÅE</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -5725,24 +5725,24 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>26 ord: - kritiskt reflektera över hur kvalitets- och säkerhetsledning organiseras och r…</t>
+          <t>35 ord: - självständigt handlägga preventivmedelsrådgivning och informera om lämpliga an…</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV2A6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3015</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>VV2002</t>
+          <t>SR3015</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>VÅE</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -5752,19 +5752,19 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>29 ord: - redogöra för gällande regelverk för olika professioner inom kommunal äldreomso…</t>
+          <t>26 ord: - kritiskt analysera, värdera, föreslå och följa upp vårdnadsinsatser och behand…</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV2002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SR3015</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>VV3006</t>
+          <t>AVV2A6</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5774,24 +5774,24 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>26 ord: - kritiskt reflektera över hur kvalitets- och säkerhetsledning organiseras och r…</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV2A6</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>VV3011</t>
+          <t>VV2002</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5801,24 +5801,24 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>19 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
+          <t>29 ord: - redogöra för gällande regelverk för olika professioner inom kommunal äldreomso…</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV2002</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>VV3012</t>
+          <t>VV3006</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5828,24 +5828,24 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>29 ord: - tillämpa adekvat vetenskaplig design och metod i datainsamling och analys samt…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3006</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>VV3012</t>
+          <t>VV3011</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5855,24 +5855,24 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>29 ord: - analysera och värdera resultat i relation till tidigare forskning samt den kli…</t>
+          <t>19 lärandemål (maximum rekommenderat: 10 för 15 hp)</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3011</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>VV3017</t>
+          <t>VV3012</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5892,14 +5892,14 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3012</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>VV3017</t>
+          <t>VV3012</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3012</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>26 ord: - göra relevanta bedömningar på mikro-, meso- och makronivå med hänsyn till samh…</t>
+          <t>29 ord: - tillämpa adekvat vetenskaplig design och metod i datainsamling och analys samt…</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
@@ -5953,86 +5953,140 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>FHV0001</t>
+          <t>VV3017</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>VÅRDVETS</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+          <t>29 ord: - analysera och värdera resultat i relation till tidigare forskning samt den kli…</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>FHV0002</t>
+          <t>VV3017</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>VÅRDVETS</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>0 lärandemål (minimum rekommenderat: 3 för 7.5 hp)</t>
+          <t>26 ord: - göra relevanta bedömningar på mikro-, meso- och makronivå med hänsyn till samh…</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=VV3017</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
+          <t>FHV0001</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>VÅRDVETS</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>För många mål</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>FHV0002</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>VÅRDVETS</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>För få mål</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>0 lärandemål (minimum rekommenderat: 3 för 7.5 hp)</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0002</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
           <t>FHV0003</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr">
+      <c r="B209" t="inlineStr">
         <is>
           <t>VÅRDVETS</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr">
+      <c r="C209" t="inlineStr">
         <is>
           <t>För få mål</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr">
+      <c r="D209" t="inlineStr">
         <is>
           <t>0 lärandemål (minimum rekommenderat: 3 för 7.5 hp)</t>
         </is>
       </c>
-      <c r="E207" s="2" t="inlineStr">
+      <c r="E209" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FHV0003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E207"/>
+  <autoFilter ref="A1:E209"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -6446,6 +6500,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E206" r:id="rId410"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A207" r:id="rId411"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E207" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A208" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E208" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A209" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E209" r:id="rId416"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>